<commit_message>
Completed final.xlsx with discrete puts and chart
</commit_message>
<xml_diff>
--- a/xlsx/final.xlsx
+++ b/xlsx/final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keith\source\repos\xlladdins\xll_ml\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adithyah Nair\source\repos\xll_ml\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFEF4C2-697C-475C-BFC8-0C347F24602F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE54975-D4BE-4156-B739-68ECA8F4D015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22276" windowHeight="13996" xr2:uid="{9BE03A92-AE89-48A8-9E12-797A60FC8C99}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{9BE03A92-AE89-48A8-9E12-797A60FC8C99}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,9 +38,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -129,8 +126,9 @@
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
+  <metadataTypes count="2">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -141,11 +139,35 @@
       </extLst>
     </bk>
   </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
+    </bk>
+  </valueMetadata>
 </metadata>
 </file>
 
@@ -333,6 +355,1537 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Strike vs Put values</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>normal_put</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$J$6:$J$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>98</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>109</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>120</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$K$6:$K$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>3.9914343421845189E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.7008934088098151E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.0058534547871929E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.11061799019468133</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.15048353300942274</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.20168732797265765</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.26648097458621844</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.34730740212793787</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.44676133725329414</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.56753930674006803</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.71238089607367172</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.88400364647703356</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0850344779622993</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.3179408286409817</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.5849647756893894</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.8880632480607282</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.2288570738163145</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.6085910627585847</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.0281066582734937</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3.4878279587501879</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>3.987761167674492</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4.5275068370385512</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>5.1062836665495652</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>5.7229621445706016</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>6.376105985444056</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>7.0640191378988391</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>7.7847961044341929</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8.5363734057617648</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>9.3165802243033653</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>10.123186539019287</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>10.953947391857227</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>11.806642276452777</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>12.679108988059141</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>13.569271600088328</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>14.47516252219144</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>15.394938837716396</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>16.326893309710854</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>17.269460583629098</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>18.221219204170339</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>19.180890108309015</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>20.14733226325697</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-406F-4560-B385-0401BE3EFE52}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$L$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>discrete_put</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$J$6:$J$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>98</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>109</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>120</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$L$6:$L$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>3.4047379960682522E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.4789567460682522E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.5531754960682522E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9.6806891217839031E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.15149439121783903</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.20618189121783903</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.26086939121783903</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.31555689121783903</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.40788732068490319</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.57976232068490319</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.75163732068490319</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.92351232068490319</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0953873206849032</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.2672623206849032</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.561530627262492</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.938483752262492</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.315436877262492</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.692390002262492</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.069343127262492</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3.446296252262492</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>3.9459687470320333</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4.5690156220320333</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>5.1920624970320333</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>5.8151093720320333</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>6.4381562470320333</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>7.0612031220320333</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>7.6847395769465408</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8.5128645769465408</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>9.3409895769465408</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>10.169114576946541</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>10.997239576946541</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>11.825364576946541</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>12.653489576946541</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>13.49122085642486</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>14.43653335642486</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>15.38184585642486</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>16.32715835642486</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>17.27247085642486</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>18.21778335642486</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>19.16309585642486</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>20.10840835642486</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-406F-4560-B385-0401BE3EFE52}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1214146496"/>
+        <c:axId val="1214164736"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1214146496"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1214164736"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1214164736"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1214146496"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>23812</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>404812</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BAA25DBC-E0B6-B5D3-4100-E7F6CA00D957}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <rv s="0">
+    <v>10</v>
+    <v>8</v>
+    <v>0</v>
+    <v>1</v>
+  </rv>
+  <rv s="1">
+    <v>8</v>
+    <v>1</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <s t="_error">
+    <k n="colOffset" t="i"/>
+    <k n="errorType" t="i"/>
+    <k n="rwOffset" t="i"/>
+    <k n="subType" t="i"/>
+  </s>
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="propagated" t="b"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -652,15 +2205,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9333FE1-19FB-4A1D-86C4-C34A7A2ACCE3}">
-  <dimension ref="B2:N46"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="B2:O216"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.578125" customWidth="1"/>
-    <col min="7" max="7" width="11.68359375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.3671875" customWidth="1"/>
+    <col min="1" max="1" width="3.59765625" customWidth="1"/>
+    <col min="6" max="6" width="15.09765625" customWidth="1"/>
+    <col min="7" max="7" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -670,13 +2224,16 @@
       <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3" cm="1">
+        <f t="array" ref="F2">_xll.\OPTION.DISCRETE(D5:D15,C5:C15)</f>
+        <v>1946882622992</v>
+      </c>
       <c r="G2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H2" s="3" cm="1">
         <f t="array" ref="H2">_xll.\OPTION.NORMAL()</f>
-        <v>1490952485744</v>
+        <v>1946833568992</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>5</v>
@@ -685,7 +2242,11 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="F3" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="F3" ca="1">_xll.OPTION.DISCRETE.XI(F2)</f>
+        <v>#VALUE!</v>
+      </c>
       <c r="I3" s="2" t="s">
         <v>6</v>
       </c>
@@ -693,7 +2254,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C4" s="1" t="s">
         <v>1</v>
       </c>
@@ -707,7 +2268,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" cm="1">
         <f t="array" ref="B5:B15">_xlfn.SEQUENCE(n+1,1,0)</f>
         <v>0</v>
@@ -730,7 +2291,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>1</v>
       </c>
@@ -751,8 +2312,12 @@
         <f t="array" ref="K6:K46">_xlfn.MAP(_xlfn.ANCHORARRAY(J6),_xlfn.LAMBDA(_xlpm.k,_xll.OPTION.BLACK.PUT(f,s,_xlpm.k,normal)))</f>
         <v>3.9914343421845189E-2</v>
       </c>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L6" cm="1">
+        <f t="array" ref="L6:L46">_xlfn.MAP(_xlfn.ANCHORARRAY(J6),_xlfn.LAMBDA(_xlpm.k,_xll.OPTION.BLACK.PUT(f,s,_xlpm.k,discrete)))</f>
+        <v>3.4047379960682522E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>2</v>
       </c>
@@ -771,8 +2336,11 @@
       <c r="K7">
         <v>5.7008934088098151E-2</v>
       </c>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L7">
+        <v>4.4789567460682522E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>3</v>
       </c>
@@ -791,8 +2359,11 @@
       <c r="K8">
         <v>8.0058534547871929E-2</v>
       </c>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L8">
+        <v>5.5531754960682522E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>4</v>
       </c>
@@ -808,8 +2379,11 @@
       <c r="K9">
         <v>0.11061799019468133</v>
       </c>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L9">
+        <v>9.6806891217839031E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>5</v>
       </c>
@@ -825,8 +2399,11 @@
       <c r="K10">
         <v>0.15048353300942274</v>
       </c>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L10">
+        <v>0.15149439121783903</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>6</v>
       </c>
@@ -842,8 +2419,11 @@
       <c r="K11">
         <v>0.20168732797265765</v>
       </c>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L11">
+        <v>0.20618189121783903</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>7</v>
       </c>
@@ -859,8 +2439,11 @@
       <c r="K12">
         <v>0.26648097458621844</v>
       </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L12">
+        <v>0.26086939121783903</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>8</v>
       </c>
@@ -876,8 +2459,11 @@
       <c r="K13">
         <v>0.34730740212793787</v>
       </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L13">
+        <v>0.31555689121783903</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>9</v>
       </c>
@@ -893,8 +2479,11 @@
       <c r="K14">
         <v>0.44676133725329414</v>
       </c>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L14">
+        <v>0.40788732068490319</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>10</v>
       </c>
@@ -910,257 +2499,360 @@
       <c r="K15">
         <v>0.56753930674006803</v>
       </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="L15">
+        <v>0.57976232068490319</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="J16">
         <v>90</v>
       </c>
       <c r="K16">
         <v>0.71238089607367172</v>
       </c>
-    </row>
-    <row r="17" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L16">
+        <v>0.75163732068490319</v>
+      </c>
+    </row>
+    <row r="17" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J17">
         <v>91</v>
       </c>
       <c r="K17">
         <v>0.88400364647703356</v>
       </c>
-    </row>
-    <row r="18" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L17">
+        <v>0.92351232068490319</v>
+      </c>
+    </row>
+    <row r="18" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J18">
         <v>92</v>
       </c>
       <c r="K18">
         <v>1.0850344779622993</v>
       </c>
-    </row>
-    <row r="19" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L18">
+        <v>1.0953873206849032</v>
+      </c>
+    </row>
+    <row r="19" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J19">
         <v>93</v>
       </c>
       <c r="K19">
         <v>1.3179408286409817</v>
       </c>
-    </row>
-    <row r="20" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L19">
+        <v>1.2672623206849032</v>
+      </c>
+    </row>
+    <row r="20" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J20">
         <v>94</v>
       </c>
       <c r="K20">
         <v>1.5849647756893894</v>
       </c>
-    </row>
-    <row r="21" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L20">
+        <v>1.561530627262492</v>
+      </c>
+    </row>
+    <row r="21" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J21">
         <v>95</v>
       </c>
       <c r="K21">
         <v>1.8880632480607282</v>
       </c>
-    </row>
-    <row r="22" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L21">
+        <v>1.938483752262492</v>
+      </c>
+    </row>
+    <row r="22" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J22">
         <v>96</v>
       </c>
       <c r="K22">
         <v>2.2288570738163145</v>
       </c>
-    </row>
-    <row r="23" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L22">
+        <v>2.315436877262492</v>
+      </c>
+    </row>
+    <row r="23" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J23">
         <v>97</v>
       </c>
       <c r="K23">
         <v>2.6085910627585847</v>
       </c>
-    </row>
-    <row r="24" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L23">
+        <v>2.692390002262492</v>
+      </c>
+    </row>
+    <row r="24" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J24">
         <v>98</v>
       </c>
       <c r="K24">
         <v>3.0281066582734937</v>
       </c>
-    </row>
-    <row r="25" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L24">
+        <v>3.069343127262492</v>
+      </c>
+    </row>
+    <row r="25" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J25">
         <v>99</v>
       </c>
       <c r="K25">
         <v>3.4878279587501879</v>
       </c>
-    </row>
-    <row r="26" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L25">
+        <v>3.446296252262492</v>
+      </c>
+    </row>
+    <row r="26" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J26">
         <v>100</v>
       </c>
       <c r="K26">
         <v>3.987761167674492</v>
       </c>
-    </row>
-    <row r="27" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L26">
+        <v>3.9459687470320333</v>
+      </c>
+    </row>
+    <row r="27" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J27">
         <v>101</v>
       </c>
       <c r="K27">
         <v>4.5275068370385512</v>
       </c>
-    </row>
-    <row r="28" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L27">
+        <v>4.5690156220320333</v>
+      </c>
+    </row>
+    <row r="28" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J28">
         <v>102</v>
       </c>
       <c r="K28">
         <v>5.1062836665495652</v>
       </c>
-    </row>
-    <row r="29" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L28">
+        <v>5.1920624970320333</v>
+      </c>
+    </row>
+    <row r="29" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J29">
         <v>103</v>
       </c>
       <c r="K29">
         <v>5.7229621445706016</v>
       </c>
-    </row>
-    <row r="30" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L29">
+        <v>5.8151093720320333</v>
+      </c>
+    </row>
+    <row r="30" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J30">
         <v>104</v>
       </c>
       <c r="K30">
         <v>6.376105985444056</v>
       </c>
-    </row>
-    <row r="31" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L30">
+        <v>6.4381562470320333</v>
+      </c>
+    </row>
+    <row r="31" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J31">
         <v>105</v>
       </c>
       <c r="K31">
         <v>7.0640191378988391</v>
       </c>
-    </row>
-    <row r="32" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L31">
+        <v>7.0612031220320333</v>
+      </c>
+    </row>
+    <row r="32" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J32">
         <v>106</v>
       </c>
       <c r="K32">
         <v>7.7847961044341929</v>
       </c>
-    </row>
-    <row r="33" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L32">
+        <v>7.6847395769465408</v>
+      </c>
+    </row>
+    <row r="33" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J33">
         <v>107</v>
       </c>
       <c r="K33">
         <v>8.5363734057617648</v>
       </c>
-    </row>
-    <row r="34" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L33">
+        <v>8.5128645769465408</v>
+      </c>
+    </row>
+    <row r="34" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J34">
         <v>108</v>
       </c>
       <c r="K34">
         <v>9.3165802243033653</v>
       </c>
-    </row>
-    <row r="35" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L34">
+        <v>9.3409895769465408</v>
+      </c>
+    </row>
+    <row r="35" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J35">
         <v>109</v>
       </c>
       <c r="K35">
         <v>10.123186539019287</v>
       </c>
-    </row>
-    <row r="36" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L35">
+        <v>10.169114576946541</v>
+      </c>
+    </row>
+    <row r="36" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J36">
         <v>110</v>
       </c>
       <c r="K36">
         <v>10.953947391857227</v>
       </c>
-    </row>
-    <row r="37" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L36">
+        <v>10.997239576946541</v>
+      </c>
+    </row>
+    <row r="37" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J37">
         <v>111</v>
       </c>
       <c r="K37">
         <v>11.806642276452777</v>
       </c>
-    </row>
-    <row r="38" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L37">
+        <v>11.825364576946541</v>
+      </c>
+    </row>
+    <row r="38" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J38">
         <v>112</v>
       </c>
       <c r="K38">
         <v>12.679108988059141</v>
       </c>
-    </row>
-    <row r="39" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L38">
+        <v>12.653489576946541</v>
+      </c>
+    </row>
+    <row r="39" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J39">
         <v>113</v>
       </c>
       <c r="K39">
         <v>13.569271600088328</v>
       </c>
-    </row>
-    <row r="40" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L39">
+        <v>13.49122085642486</v>
+      </c>
+    </row>
+    <row r="40" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J40">
         <v>114</v>
       </c>
       <c r="K40">
         <v>14.47516252219144</v>
       </c>
-    </row>
-    <row r="41" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L40">
+        <v>14.43653335642486</v>
+      </c>
+    </row>
+    <row r="41" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J41">
         <v>115</v>
       </c>
       <c r="K41">
         <v>15.394938837716396</v>
       </c>
-    </row>
-    <row r="42" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L41">
+        <v>15.38184585642486</v>
+      </c>
+    </row>
+    <row r="42" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J42">
         <v>116</v>
       </c>
       <c r="K42">
         <v>16.326893309710854</v>
       </c>
-    </row>
-    <row r="43" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L42">
+        <v>16.32715835642486</v>
+      </c>
+    </row>
+    <row r="43" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J43">
         <v>117</v>
       </c>
       <c r="K43">
         <v>17.269460583629098</v>
       </c>
-    </row>
-    <row r="44" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L43">
+        <v>17.27247085642486</v>
+      </c>
+    </row>
+    <row r="44" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J44">
         <v>118</v>
       </c>
       <c r="K44">
         <v>18.221219204170339</v>
       </c>
-    </row>
-    <row r="45" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L44">
+        <v>18.21778335642486</v>
+      </c>
+    </row>
+    <row r="45" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J45">
         <v>119</v>
       </c>
       <c r="K45">
         <v>19.180890108309015</v>
       </c>
-    </row>
-    <row r="46" spans="10:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="L45">
+        <v>19.16309585642486</v>
+      </c>
+    </row>
+    <row r="46" spans="10:12" x14ac:dyDescent="0.3">
       <c r="J46">
         <v>120</v>
       </c>
       <c r="K46">
         <v>20.14733226325697</v>
       </c>
+      <c r="L46">
+        <v>20.10840835642486</v>
+      </c>
+    </row>
+    <row r="216" spans="15:15" x14ac:dyDescent="0.3">
+      <c r="O216" t="e" vm="2">
+        <f ca="1">AVERAGE(_xlfn.ANCHORARRAY(F3))</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>